<commit_message>
arrumando bacia e sub-bacia
</commit_message>
<xml_diff>
--- a/integracao.xlsx
+++ b/integracao.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="59">
   <si>
     <t>propietario</t>
   </si>
@@ -186,9 +186,6 @@
     <t>inserido no bioma amazonico?</t>
   </si>
   <si>
-    <t>11.111.111/1111-78</t>
-  </si>
-  <si>
     <t>casado(a)</t>
   </si>
   <si>
@@ -199,6 +196,18 @@
   </si>
   <si>
     <t>cpf</t>
+  </si>
+  <si>
+    <t>32.251.489/5614-55</t>
+  </si>
+  <si>
+    <t>bacia</t>
+  </si>
+  <si>
+    <t>sub-bacia</t>
+  </si>
+  <si>
+    <t>Rio tocantins</t>
   </si>
 </sst>
 </file>
@@ -669,7 +678,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="B1:F24"/>
+  <dimension ref="B1:F26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.42578125" customWidth="1"/>
@@ -702,7 +711,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="6" t="s">
@@ -740,7 +749,7 @@
         <v>20</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>24</v>
@@ -775,7 +784,7 @@
         <v>41</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -786,7 +795,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F10" s="18" t="s">
         <v>47</v>
@@ -800,7 +809,7 @@
         <v>1234.5123000000001</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F11" s="15" t="s">
         <v>43</v>
@@ -814,7 +823,7 @@
         <v>156.65</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F12" s="15"/>
     </row>
@@ -826,7 +835,7 @@
         <v>25000000</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F13" s="4"/>
     </row>
@@ -918,14 +927,29 @@
         <v>47</v>
       </c>
     </row>
+    <row r="25" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="10"/>
+    </row>
   </sheetData>
-  <dataValidations xWindow="919" yWindow="330" count="6">
+  <dataValidations xWindow="919" yWindow="330" count="7">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="utilize apenas 2 letras e deixe-as maiusculo" sqref="C20"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="deixe no formato 00/00/0000" sqref="F8 F6 F4"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="deixe no formata de cpf ou cnpj_x000a__x000a_000.000.000-00_x000a__x000a_00.000.000/0000-00" sqref="C3 C6"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="deixe no formatado com estado : cidade - uf" sqref="F5 F3"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="NESTE CAMPO VOCE UTILIZE VIRGULAS E NÃO PONTOS" sqref="C11 C17 C18"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="não precisa responder esses dados se não for casado(a)" sqref="F12 F13"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="se não houver sub-bacia voce pode deixar em branco mesmo" sqref="C26"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>